<commit_message>
Filing cabinet included for every customer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cpjf5ajPeXVSvyknWthQ2
</commit_message>
<xml_diff>
--- a/content/downloads/Battenkill-Ag-H2A-Audit-Checklist.xlsx
+++ b/content/downloads/Battenkill-Ag-H2A-Audit-Checklist.xlsx
@@ -251,7 +251,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -515,6 +515,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -823,7 +827,7 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="41">
-      <c r="B6" s="46" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
         <is>
           <t>1. Fill in the Season Info tab once per season (farm name, case number, certification date).</t>
         </is>
@@ -837,21 +841,21 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="41">
-      <c r="B8" s="46" t="inlineStr">
+      <c r="B8" s="48" t="inlineStr">
         <is>
           <t>3. Write where each record is kept (binder, folder, payroll system) so anyone on your team can find it fast.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="41">
-      <c r="B9" s="46" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>4. Use the Worker Departures tab any time a worker abandons the job or is fired for cause. It works out the 2-working-day notice deadline for you.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="41">
-      <c r="B10" s="46" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>5. Click any Rule to read the regulation, or any Learn more link for a plain-English guide. The Resources tab lists more help by topic, like housing, wages and travel.</t>
         </is>
@@ -872,14 +876,14 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="41">
-      <c r="B13" s="46" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>Light yellow cells are for you to fill in. Everything else calculates on its own.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="41">
-      <c r="B14" s="46" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>Rows in grey italics are examples showing the expected format. Overwrite or delete them.</t>
         </is>
@@ -896,9 +900,9 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="41">
-      <c r="B17" s="46" t="inlineStr">
-        <is>
-          <t>Battenkill Ag customers can add a digital filing cabinet that tracks these records automatically, organized by requirement, so an audit response starts from a complete folder.</t>
+      <c r="B17" s="48" t="inlineStr">
+        <is>
+          <t>Every Battenkill Ag customer gets a digital filing cabinet to keep track of important documents, deadlines and billing, with these records organized by requirement, so an audit response starts from a complete folder.</t>
         </is>
       </c>
     </row>
@@ -1151,42 +1155,42 @@
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1" s="41">
-      <c r="A8" s="62" t="inlineStr">
+      <c r="A8" s="63" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="63" t="inlineStr">
         <is>
           <t>Record</t>
         </is>
       </c>
-      <c r="C8" s="62" t="inlineStr">
+      <c r="C8" s="63" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="D8" s="62" t="inlineStr">
+      <c r="D8" s="63" t="inlineStr">
         <is>
           <t>Applies to my farm?</t>
         </is>
       </c>
-      <c r="E8" s="62" t="inlineStr">
+      <c r="E8" s="63" t="inlineStr">
         <is>
           <t>Have it?</t>
         </is>
       </c>
-      <c r="F8" s="62" t="inlineStr">
+      <c r="F8" s="63" t="inlineStr">
         <is>
           <t>Where it's kept</t>
         </is>
       </c>
-      <c r="G8" s="62" t="inlineStr">
+      <c r="G8" s="63" t="inlineStr">
         <is>
           <t>Last updated</t>
         </is>
       </c>
-      <c r="H8" s="62" t="inlineStr">
+      <c r="H8" s="63" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2097,7 +2101,7 @@
           <t>Notices to workers about any delay in your start date</t>
         </is>
       </c>
-      <c r="C45" s="70" t="inlineStr">
+      <c r="C45" s="71" t="inlineStr">
         <is>
           <t>Job order</t>
         </is>
@@ -2170,7 +2174,7 @@
     </row>
     <row r="49" s="41">
       <c r="A49" s="75" t="n"/>
-      <c r="B49" s="76" t="inlineStr">
+      <c r="B49" s="91" t="inlineStr">
         <is>
           <t>Click any Rule to read the regulation, or any Learn more link for a plain-English guide. More links are on the Resources tab.</t>
         </is>
@@ -2185,9 +2189,9 @@
     </row>
     <row r="50" s="41">
       <c r="A50" s="75" t="n"/>
-      <c r="B50" s="76" t="inlineStr">
-        <is>
-          <t>Battenkill Ag customers can add a digital filing cabinet that tracks every record on this list automatically.</t>
+      <c r="B50" s="91" t="inlineStr">
+        <is>
+          <t>Every Battenkill Ag customer gets a digital filing cabinet to keep track of important documents, deadlines and billing, including every record on this list.</t>
         </is>
       </c>
       <c r="C50" s="75" t="n"/>
@@ -2200,7 +2204,7 @@
     </row>
     <row r="51" s="41">
       <c r="A51" s="75" t="n"/>
-      <c r="B51" s="76" t="inlineStr">
+      <c r="B51" s="91" t="inlineStr">
         <is>
           <t>General information, not legal advice. Your case may require records not listed here.</t>
         </is>
@@ -2449,42 +2453,42 @@
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1" s="41">
-      <c r="A5" s="62" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>Worker name</t>
         </is>
       </c>
-      <c r="B5" s="62" t="inlineStr">
+      <c r="B5" s="63" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="C5" s="62" t="inlineStr">
+      <c r="C5" s="63" t="inlineStr">
         <is>
           <t>Abandonment or termination date</t>
         </is>
       </c>
-      <c r="D5" s="62" t="inlineStr">
+      <c r="D5" s="63" t="inlineStr">
         <is>
           <t>Notice due (2 working days)</t>
         </is>
       </c>
-      <c r="E5" s="62" t="inlineStr">
+      <c r="E5" s="63" t="inlineStr">
         <is>
           <t>Date DOL notified</t>
         </is>
       </c>
-      <c r="F5" s="62" t="inlineStr">
+      <c r="F5" s="63" t="inlineStr">
         <is>
           <t>Date DHS notified</t>
         </is>
       </c>
-      <c r="G5" s="62" t="inlineStr">
+      <c r="G5" s="63" t="inlineStr">
         <is>
           <t>On time?</t>
         </is>
       </c>
-      <c r="H5" s="62" t="inlineStr">
+      <c r="H5" s="63" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3381,7 +3385,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="90" t="inlineStr">
+      <c r="A29" s="92" t="inlineStr">
         <is>
           <t>Questions? Battenkill Ag Services  |  512-540-4533  |  max@battenkillag.com  |  www.battenkillag.com</t>
         </is>

</xml_diff>